<commit_message>
docs: sprint 6 artifacts
</commit_message>
<xml_diff>
--- a/docs/Requirements_Stack.xlsx
+++ b/docs/Requirements_Stack.xlsx
@@ -335,7 +335,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F38"/>
+  <dimension ref="B2:F47"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="8.710000000000001" customWidth="1" style="4" min="1" max="2"/>
@@ -925,40 +925,40 @@
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1" s="4">
-      <c r="B32" t="n">
+      <c r="B32" s="0" t="n">
         <v>30</v>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="0" t="inlineStr">
         <is>
           <t>Spike: Research React Native/Expo for mobile migration</t>
         </is>
       </c>
-      <c r="D32" t="n">
-        <v>3</v>
-      </c>
-      <c r="E32" t="n">
+      <c r="D32" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="E32" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="F32" t="n">
+      <c r="F32" s="0" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="33" ht="14.25" customHeight="1" s="4">
-      <c r="B33" t="n">
+      <c r="B33" s="0" t="n">
         <v>31</v>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="0" t="inlineStr">
         <is>
           <t>Initialize Expo React Native project</t>
         </is>
       </c>
-      <c r="D33" t="n">
-        <v>5</v>
-      </c>
-      <c r="E33" t="n">
+      <c r="D33" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="E33" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="F33" t="n">
+      <c r="F33" s="0" t="n">
         <v>5</v>
       </c>
     </row>
@@ -977,26 +977,26 @@
       <c r="E34" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="F34" t="n">
+      <c r="F34" s="0" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1" s="4">
-      <c r="B35" t="n">
+      <c r="B35" s="0" t="n">
         <v>33</v>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="0" t="inlineStr">
         <is>
           <t>Fetch and display nearby restaurants on map (mobile)</t>
         </is>
       </c>
-      <c r="D35" t="n">
+      <c r="D35" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="E35" t="n">
-        <v>3</v>
-      </c>
-      <c r="F35" t="n">
+      <c r="E35" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="F35" s="0" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1015,57 +1015,219 @@
       <c r="E36" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="F36" t="n">
+      <c r="F36" s="0" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="37" ht="14.25" customHeight="1" s="4">
-      <c r="B37" t="n">
+      <c r="B37" s="0" t="n">
         <v>35</v>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="0" t="inlineStr">
         <is>
           <t>User authentication — login and signup (mobile)</t>
         </is>
       </c>
-      <c r="D37" t="n">
-        <v>5</v>
-      </c>
-      <c r="E37" t="n">
-        <v>5</v>
-      </c>
-      <c r="F37" t="n">
+      <c r="D37" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="E37" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="F37" s="0" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1" s="4">
-      <c r="B38" t="n">
+      <c r="B38" s="0" t="n">
         <v>36</v>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C38" s="0" t="inlineStr">
         <is>
           <t>Basic restaurant filters — cuisine, distance, price, rating (mobile)</t>
         </is>
       </c>
-      <c r="D38" t="n">
-        <v>5</v>
-      </c>
-      <c r="E38" t="n">
-        <v>5</v>
-      </c>
-      <c r="F38" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="39" ht="14.25" customHeight="1" s="4"/>
-    <row r="40" ht="14.25" customHeight="1" s="4"/>
-    <row r="41" ht="14.25" customHeight="1" s="4"/>
-    <row r="42" ht="14.25" customHeight="1" s="4"/>
-    <row r="43" ht="14.25" customHeight="1" s="4"/>
-    <row r="44" ht="14.25" customHeight="1" s="4"/>
-    <row r="45" ht="14.25" customHeight="1" s="4"/>
-    <row r="46" ht="14.25" customHeight="1" s="4"/>
-    <row r="47" ht="14.25" customHeight="1" s="4"/>
+      <c r="D38" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="E38" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="F38" s="0" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="39" ht="14.25" customHeight="1" s="4">
+      <c r="B39" t="n">
+        <v>37</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Restaurant list view (mobile)</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>5</v>
+      </c>
+      <c r="E39" t="n">
+        <v>6</v>
+      </c>
+      <c r="F39" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="40" ht="14.25" customHeight="1" s="4">
+      <c r="B40" t="n">
+        <v>38</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Sort restaurants by distance (mobile)</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>3</v>
+      </c>
+      <c r="E40" t="n">
+        <v>6</v>
+      </c>
+      <c r="F40" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="41" ht="14.25" customHeight="1" s="4">
+      <c r="B41" t="n">
+        <v>39</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Display restaurants with deals using custom marker (mobile)</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>3</v>
+      </c>
+      <c r="E41" t="n">
+        <v>6</v>
+      </c>
+      <c r="F41" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="42" ht="14.25" customHeight="1" s="4">
+      <c r="B42" t="n">
+        <v>40</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Save restaurant as favorite (mobile)</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>3</v>
+      </c>
+      <c r="E42" t="n">
+        <v>7</v>
+      </c>
+      <c r="F42" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="43" ht="14.25" customHeight="1" s="4">
+      <c r="B43" t="n">
+        <v>41</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>View list of saved favorite restaurants (mobile)</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>3</v>
+      </c>
+      <c r="E43" t="n">
+        <v>7</v>
+      </c>
+      <c r="F43" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="44" ht="14.25" customHeight="1" s="4">
+      <c r="B44" t="n">
+        <v>42</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Persist favorites in Supabase (mobile)</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>3</v>
+      </c>
+      <c r="E44" t="n">
+        <v>7</v>
+      </c>
+      <c r="F44" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="45" ht="14.25" customHeight="1" s="4">
+      <c r="B45" t="n">
+        <v>43</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>User profile screen (mobile)</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>3</v>
+      </c>
+      <c r="E45" t="n">
+        <v>7</v>
+      </c>
+      <c r="F45" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="46" ht="14.25" customHeight="1" s="4">
+      <c r="B46" t="n">
+        <v>44</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Search restaurants by name (mobile)</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>3</v>
+      </c>
+      <c r="E46" t="n">
+        <v>5</v>
+      </c>
+      <c r="F46" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="47" ht="14.25" customHeight="1" s="4">
+      <c r="B47" t="n">
+        <v>45</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Integrate deals API with restaurant data (mobile)</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>8</v>
+      </c>
+      <c r="E47" t="n">
+        <v>5</v>
+      </c>
+      <c r="F47" t="n">
+        <v>6</v>
+      </c>
+    </row>
     <row r="48" ht="14.25" customHeight="1" s="4"/>
     <row r="49" ht="14.25" customHeight="1" s="4"/>
     <row r="50" ht="14.25" customHeight="1" s="4"/>

</xml_diff>